<commit_message>
beetwen second and third week
</commit_message>
<xml_diff>
--- a/Organisation/02_Jahresplan_SJ2026_27_SPL_4AHWII.xlsx
+++ b/Organisation/02_Jahresplan_SJ2026_27_SPL_4AHWII.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dokumente\Schuldateien\SPL\Handy Garage\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dokumente\Schuldateien\SPL\Handy Garage\Organisation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCAF1778-6D0B-47EC-B4E0-2A0E286ED234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB21C77C-816D-4E6D-B07D-F9380138823A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Minutes" sheetId="1" r:id="rId1"/>
+    <sheet name="Zeitplan" sheetId="5" r:id="rId1"/>
+    <sheet name="Protokolle" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -55,12 +56,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="141">
   <si>
     <t>Monat</t>
-  </si>
-  <si>
-    <t>Thema</t>
   </si>
   <si>
     <t>Datum</t>
@@ -638,6 +636,45 @@
   <si>
     <t>Protokolle\Protokoll 11.09.2026.docx</t>
   </si>
+  <si>
+    <t>1) Projektstart</t>
+  </si>
+  <si>
+    <t>2) Produktidee</t>
+  </si>
+  <si>
+    <t>3)Übersicht aller Funktionseinheiten</t>
+  </si>
+  <si>
+    <t>5)Status Gesamtkonzept</t>
+  </si>
+  <si>
+    <t>Technische Dokumentation</t>
+  </si>
+  <si>
+    <t>Projekt Wochen</t>
+  </si>
+  <si>
+    <t>KW</t>
+  </si>
+  <si>
+    <t>4) Alle FE einzeln funktionsfähig</t>
+  </si>
+  <si>
+    <t>6) Finales Produkt</t>
+  </si>
+  <si>
+    <t>Notizen</t>
+  </si>
+  <si>
+    <t>SPL Wochen</t>
+  </si>
+  <si>
+    <t>Meilenstein Professor</t>
+  </si>
+  <si>
+    <t>..\Protokolle\Protokoll 18.09.2026.docx</t>
+  </si>
 </sst>
 </file>
 
@@ -647,7 +684,7 @@
     <numFmt numFmtId="164" formatCode="ddd\,\ d\.\ mmm\ yyyy"/>
     <numFmt numFmtId="165" formatCode="mmmm"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -670,8 +707,12 @@
       <color theme="10"/>
       <name val="Helvetica Neue"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Helvetica Neue"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -720,8 +761,26 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="28">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -1021,36 +1080,6 @@
       <top style="thin">
         <color indexed="8"/>
       </top>
-      <bottom style="medium">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="medium">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
       <bottom style="dotted">
         <color indexed="8"/>
       </bottom>
@@ -1116,6 +1145,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
@@ -1125,7 +1169,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1142,12 +1186,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1159,9 +1197,6 @@
     <xf numFmtId="49" fontId="1" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1237,47 +1272,95 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="23" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="10" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="26" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="26" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="10" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1285,20 +1368,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2427,24 +2498,676 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CC0EE35-C06D-4973-84FF-C57664B42531}">
+  <dimension ref="B2:I32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2"/>
+  <cols>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" ht="18.600000000000001" customHeight="1">
+      <c r="B2" s="58" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" s="58" t="s">
+        <v>134</v>
+      </c>
+      <c r="E2" s="61" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="61" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="61" t="s">
+        <v>139</v>
+      </c>
+      <c r="H2" s="61" t="s">
+        <v>137</v>
+      </c>
+      <c r="I2" s="61" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9">
+      <c r="B3" s="60">
+        <v>1</v>
+      </c>
+      <c r="C3" s="59">
+        <v>1</v>
+      </c>
+      <c r="D3" s="48" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="62" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="50">
+        <v>46276</v>
+      </c>
+      <c r="G3" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="H3" s="52"/>
+      <c r="I3" s="53"/>
+    </row>
+    <row r="4" spans="2:9">
+      <c r="B4" s="60">
+        <v>2</v>
+      </c>
+      <c r="C4" s="59">
+        <v>2</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="62"/>
+      <c r="F4" s="50">
+        <f t="shared" ref="F4:F32" si="0">$F$3+(C4-1)*7</f>
+        <v>46283</v>
+      </c>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="55"/>
+    </row>
+    <row r="5" spans="2:9">
+      <c r="B5" s="60">
+        <v>3</v>
+      </c>
+      <c r="C5" s="59">
+        <v>3</v>
+      </c>
+      <c r="D5" s="48" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="62"/>
+      <c r="F5" s="50">
+        <f t="shared" si="0"/>
+        <v>46290</v>
+      </c>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="55"/>
+    </row>
+    <row r="6" spans="2:9">
+      <c r="B6" s="60">
+        <v>4</v>
+      </c>
+      <c r="C6" s="59">
+        <v>4</v>
+      </c>
+      <c r="D6" s="48" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="50">
+        <f t="shared" si="0"/>
+        <v>46297</v>
+      </c>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="55"/>
+    </row>
+    <row r="7" spans="2:9">
+      <c r="B7" s="60">
+        <v>5</v>
+      </c>
+      <c r="C7" s="59">
+        <v>5</v>
+      </c>
+      <c r="D7" s="48" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="62"/>
+      <c r="F7" s="50">
+        <f t="shared" si="0"/>
+        <v>46304</v>
+      </c>
+      <c r="G7" s="51" t="s">
+        <v>129</v>
+      </c>
+      <c r="H7" s="54"/>
+      <c r="I7" s="55"/>
+    </row>
+    <row r="8" spans="2:9">
+      <c r="B8" s="60">
+        <v>6</v>
+      </c>
+      <c r="C8" s="59">
+        <v>6</v>
+      </c>
+      <c r="D8" s="48" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="62"/>
+      <c r="F8" s="50">
+        <f t="shared" si="0"/>
+        <v>46311</v>
+      </c>
+      <c r="G8" s="54"/>
+      <c r="H8" s="54"/>
+      <c r="I8" s="55"/>
+    </row>
+    <row r="9" spans="2:9">
+      <c r="B9" s="60">
+        <v>7</v>
+      </c>
+      <c r="C9" s="59">
+        <v>7</v>
+      </c>
+      <c r="D9" s="48" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="62"/>
+      <c r="F9" s="50">
+        <f t="shared" si="0"/>
+        <v>46318</v>
+      </c>
+      <c r="G9" s="54"/>
+      <c r="H9" s="54"/>
+      <c r="I9" s="55"/>
+    </row>
+    <row r="10" spans="2:9">
+      <c r="B10" s="60">
+        <v>8</v>
+      </c>
+      <c r="C10" s="59">
+        <v>9</v>
+      </c>
+      <c r="D10" s="48" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="62" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="50">
+        <f t="shared" si="0"/>
+        <v>46332</v>
+      </c>
+      <c r="G10" s="54"/>
+      <c r="H10" s="54"/>
+      <c r="I10" s="53"/>
+    </row>
+    <row r="11" spans="2:9">
+      <c r="B11" s="60">
+        <v>9</v>
+      </c>
+      <c r="C11" s="59">
+        <v>10</v>
+      </c>
+      <c r="D11" s="48" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="62"/>
+      <c r="F11" s="50">
+        <f t="shared" si="0"/>
+        <v>46339</v>
+      </c>
+      <c r="G11" s="51" t="s">
+        <v>130</v>
+      </c>
+      <c r="H11" s="54"/>
+      <c r="I11" s="55"/>
+    </row>
+    <row r="12" spans="2:9">
+      <c r="B12" s="60">
+        <v>10</v>
+      </c>
+      <c r="C12" s="59">
+        <v>11</v>
+      </c>
+      <c r="D12" s="48" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="62"/>
+      <c r="F12" s="50">
+        <f t="shared" si="0"/>
+        <v>46346</v>
+      </c>
+      <c r="G12" s="47"/>
+      <c r="H12" s="54"/>
+      <c r="I12" s="55"/>
+    </row>
+    <row r="13" spans="2:9">
+      <c r="B13" s="60">
+        <v>11</v>
+      </c>
+      <c r="C13" s="59">
+        <v>13</v>
+      </c>
+      <c r="D13" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="62" t="s">
+        <v>42</v>
+      </c>
+      <c r="F13" s="50">
+        <f t="shared" si="0"/>
+        <v>46360</v>
+      </c>
+      <c r="G13" s="54"/>
+      <c r="H13" s="54"/>
+      <c r="I13" s="55"/>
+    </row>
+    <row r="14" spans="2:9">
+      <c r="B14" s="60">
+        <v>12</v>
+      </c>
+      <c r="C14" s="59">
+        <v>14</v>
+      </c>
+      <c r="D14" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="62"/>
+      <c r="F14" s="50">
+        <f t="shared" si="0"/>
+        <v>46367</v>
+      </c>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="53"/>
+    </row>
+    <row r="15" spans="2:9">
+      <c r="B15" s="60">
+        <v>13</v>
+      </c>
+      <c r="C15" s="59">
+        <v>15</v>
+      </c>
+      <c r="D15" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="62"/>
+      <c r="F15" s="50">
+        <f t="shared" si="0"/>
+        <v>46374</v>
+      </c>
+      <c r="G15" s="54"/>
+      <c r="H15" s="54"/>
+      <c r="I15" s="53"/>
+    </row>
+    <row r="16" spans="2:9">
+      <c r="B16" s="60">
+        <v>14</v>
+      </c>
+      <c r="C16" s="59">
+        <v>19</v>
+      </c>
+      <c r="D16" s="48" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="62"/>
+      <c r="F16" s="50">
+        <f t="shared" si="0"/>
+        <v>46402</v>
+      </c>
+      <c r="G16" s="51" t="s">
+        <v>135</v>
+      </c>
+      <c r="H16" s="54"/>
+      <c r="I16" s="55"/>
+    </row>
+    <row r="17" spans="2:9">
+      <c r="B17" s="60">
+        <v>15</v>
+      </c>
+      <c r="C17" s="59">
+        <v>20</v>
+      </c>
+      <c r="D17" s="48" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="62"/>
+      <c r="F17" s="50">
+        <f t="shared" si="0"/>
+        <v>46409</v>
+      </c>
+      <c r="G17" s="54"/>
+      <c r="H17" s="54"/>
+      <c r="I17" s="56"/>
+    </row>
+    <row r="18" spans="2:9">
+      <c r="B18" s="60">
+        <v>16</v>
+      </c>
+      <c r="C18" s="59">
+        <v>21</v>
+      </c>
+      <c r="D18" s="48" t="s">
+        <v>62</v>
+      </c>
+      <c r="E18" s="62"/>
+      <c r="F18" s="50">
+        <f t="shared" si="0"/>
+        <v>46416</v>
+      </c>
+      <c r="G18" s="54"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="53"/>
+    </row>
+    <row r="19" spans="2:9">
+      <c r="B19" s="60">
+        <v>17</v>
+      </c>
+      <c r="C19" s="59">
+        <v>23</v>
+      </c>
+      <c r="D19" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="E19" s="63"/>
+      <c r="F19" s="50">
+        <f t="shared" si="0"/>
+        <v>46430</v>
+      </c>
+      <c r="G19" s="57" t="s">
+        <v>131</v>
+      </c>
+      <c r="H19" s="54"/>
+      <c r="I19" s="55"/>
+    </row>
+    <row r="20" spans="2:9">
+      <c r="B20" s="60">
+        <v>18</v>
+      </c>
+      <c r="C20" s="59">
+        <v>24</v>
+      </c>
+      <c r="D20" s="48" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" s="63"/>
+      <c r="F20" s="50">
+        <f t="shared" si="0"/>
+        <v>46437</v>
+      </c>
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="55"/>
+    </row>
+    <row r="21" spans="2:9">
+      <c r="B21" s="60">
+        <v>19</v>
+      </c>
+      <c r="C21" s="59">
+        <v>25</v>
+      </c>
+      <c r="D21" s="48" t="s">
+        <v>74</v>
+      </c>
+      <c r="E21" s="63"/>
+      <c r="F21" s="50">
+        <f t="shared" si="0"/>
+        <v>46444</v>
+      </c>
+      <c r="G21" s="54"/>
+      <c r="H21" s="54"/>
+      <c r="I21" s="55"/>
+    </row>
+    <row r="22" spans="2:9">
+      <c r="B22" s="60">
+        <v>20</v>
+      </c>
+      <c r="C22" s="59">
+        <v>26</v>
+      </c>
+      <c r="D22" s="48" t="s">
+        <v>76</v>
+      </c>
+      <c r="E22" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="F22" s="50">
+        <f t="shared" si="0"/>
+        <v>46451</v>
+      </c>
+      <c r="G22" s="54"/>
+      <c r="H22" s="54"/>
+      <c r="I22" s="55"/>
+    </row>
+    <row r="23" spans="2:9">
+      <c r="B23" s="60">
+        <v>21</v>
+      </c>
+      <c r="C23" s="59">
+        <v>27</v>
+      </c>
+      <c r="D23" s="48" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23" s="62"/>
+      <c r="F23" s="50">
+        <f t="shared" si="0"/>
+        <v>46458</v>
+      </c>
+      <c r="G23" s="54"/>
+      <c r="H23" s="54"/>
+      <c r="I23" s="55"/>
+    </row>
+    <row r="24" spans="2:9">
+      <c r="B24" s="60">
+        <v>22</v>
+      </c>
+      <c r="C24" s="59">
+        <v>28</v>
+      </c>
+      <c r="D24" s="48" t="s">
+        <v>81</v>
+      </c>
+      <c r="E24" s="62"/>
+      <c r="F24" s="50">
+        <f t="shared" si="0"/>
+        <v>46465</v>
+      </c>
+      <c r="G24" s="54"/>
+      <c r="H24" s="54"/>
+      <c r="I24" s="55"/>
+    </row>
+    <row r="25" spans="2:9">
+      <c r="B25" s="60">
+        <v>23</v>
+      </c>
+      <c r="C25" s="59">
+        <v>30</v>
+      </c>
+      <c r="D25" s="48" t="s">
+        <v>86</v>
+      </c>
+      <c r="E25" s="62" t="s">
+        <v>89</v>
+      </c>
+      <c r="F25" s="50">
+        <f t="shared" si="0"/>
+        <v>46479</v>
+      </c>
+      <c r="G25" s="54"/>
+      <c r="H25" s="54"/>
+      <c r="I25" s="53"/>
+    </row>
+    <row r="26" spans="2:9">
+      <c r="B26" s="60">
+        <v>24</v>
+      </c>
+      <c r="C26" s="59">
+        <v>31</v>
+      </c>
+      <c r="D26" s="48" t="s">
+        <v>88</v>
+      </c>
+      <c r="E26" s="62"/>
+      <c r="F26" s="50">
+        <f t="shared" si="0"/>
+        <v>46486</v>
+      </c>
+      <c r="G26" s="54"/>
+      <c r="H26" s="54"/>
+      <c r="I26" s="55"/>
+    </row>
+    <row r="27" spans="2:9">
+      <c r="B27" s="60">
+        <v>25</v>
+      </c>
+      <c r="C27" s="59">
+        <v>33</v>
+      </c>
+      <c r="D27" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="E27" s="62"/>
+      <c r="F27" s="50">
+        <f t="shared" si="0"/>
+        <v>46500</v>
+      </c>
+      <c r="G27" s="54"/>
+      <c r="H27" s="54"/>
+      <c r="I27" s="55"/>
+    </row>
+    <row r="28" spans="2:9">
+      <c r="B28" s="60">
+        <v>26</v>
+      </c>
+      <c r="C28" s="59">
+        <v>34</v>
+      </c>
+      <c r="D28" s="48" t="s">
+        <v>96</v>
+      </c>
+      <c r="E28" s="62"/>
+      <c r="F28" s="50">
+        <f t="shared" si="0"/>
+        <v>46507</v>
+      </c>
+      <c r="G28" s="51" t="s">
+        <v>136</v>
+      </c>
+      <c r="H28" s="54"/>
+      <c r="I28" s="55"/>
+    </row>
+    <row r="29" spans="2:9">
+      <c r="B29" s="60">
+        <v>27</v>
+      </c>
+      <c r="C29" s="59">
+        <v>35</v>
+      </c>
+      <c r="D29" s="48" t="s">
+        <v>99</v>
+      </c>
+      <c r="E29" s="62" t="s">
+        <v>100</v>
+      </c>
+      <c r="F29" s="50">
+        <f t="shared" si="0"/>
+        <v>46514</v>
+      </c>
+      <c r="G29" s="54"/>
+      <c r="H29" s="54"/>
+      <c r="I29" s="53"/>
+    </row>
+    <row r="30" spans="2:9">
+      <c r="B30" s="60">
+        <v>28</v>
+      </c>
+      <c r="C30" s="59">
+        <v>36</v>
+      </c>
+      <c r="D30" s="48" t="s">
+        <v>103</v>
+      </c>
+      <c r="E30" s="62"/>
+      <c r="F30" s="50">
+        <f t="shared" si="0"/>
+        <v>46521</v>
+      </c>
+      <c r="G30" s="54"/>
+      <c r="H30" s="54"/>
+      <c r="I30" s="55"/>
+    </row>
+    <row r="31" spans="2:9">
+      <c r="B31" s="60">
+        <v>29</v>
+      </c>
+      <c r="C31" s="59">
+        <v>37</v>
+      </c>
+      <c r="D31" s="48" t="s">
+        <v>105</v>
+      </c>
+      <c r="E31" s="62"/>
+      <c r="F31" s="50">
+        <f t="shared" si="0"/>
+        <v>46528</v>
+      </c>
+      <c r="G31" s="54"/>
+      <c r="H31" s="54"/>
+      <c r="I31" s="53"/>
+    </row>
+    <row r="32" spans="2:9">
+      <c r="B32" s="60">
+        <v>30</v>
+      </c>
+      <c r="C32" s="59">
+        <v>39</v>
+      </c>
+      <c r="D32" s="48" t="s">
+        <v>111</v>
+      </c>
+      <c r="E32" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="F32" s="50">
+        <f t="shared" si="0"/>
+        <v>46542</v>
+      </c>
+      <c r="G32" s="57" t="s">
+        <v>132</v>
+      </c>
+      <c r="H32" s="54"/>
+      <c r="I32" s="55"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="E25:E28"/>
+    <mergeCell ref="E29:E31"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="E19:E21"/>
+  </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:J45"/>
+  <dimension ref="B1:H45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="19.95" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="6.109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="6.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" style="1" customWidth="1"/>
-    <col min="5" max="6" width="16.33203125" style="1" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="16" style="1" customWidth="1"/>
-    <col min="8" max="8" width="37.33203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="31.6640625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="43.109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="16.33203125" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="16.33203125" style="1"/>
+    <col min="4" max="4" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" style="1" customWidth="1"/>
+    <col min="6" max="6" width="37.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="32.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="43.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="16.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="44.7" customHeight="1">
+    <row r="1" spans="2:8" ht="44.7" customHeight="1">
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
       <c r="D1" s="4" t="s">
@@ -2453,1049 +3176,817 @@
       <c r="E1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="8" t="s">
+    </row>
+    <row r="2" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B2" s="7" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="D2" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="51" t="s">
+      <c r="E2" s="9">
+        <v>46276</v>
+      </c>
+      <c r="F2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="53"/>
-      <c r="F2" s="11">
-        <v>45901</v>
-      </c>
-      <c r="G2" s="12">
-        <v>46276</v>
-      </c>
-      <c r="H2" s="13" t="s">
+      <c r="G2" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="H2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="57" t="s">
-        <v>128</v>
-      </c>
-      <c r="J2" s="15" t="s">
+    </row>
+    <row r="3" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B3" s="13" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B3" s="16" t="s">
+      <c r="C3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="D3" s="65"/>
+      <c r="E3" s="9" cm="1">
+        <f t="array" ref="E3">E2+7</f>
+        <v>46283</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="46" t="s">
+        <v>140</v>
+      </c>
+      <c r="H3" s="15"/>
+    </row>
+    <row r="4" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B4" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="11" cm="1">
-        <f t="array" ref="F3">F2+7</f>
-        <v>45908</v>
-      </c>
-      <c r="G3" s="12" cm="1">
-        <f t="array" ref="G3">G2+7</f>
-        <v>46283</v>
-      </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="18"/>
-    </row>
-    <row r="4" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B4" s="16" t="s">
+      <c r="C4" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="D4" s="65"/>
+      <c r="E4" s="9" cm="1">
+        <f t="array" ref="E4">E3+7</f>
+        <v>46290</v>
+      </c>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="15"/>
+    </row>
+    <row r="5" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B5" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="11" cm="1">
-        <f t="array" ref="F4">F3+7</f>
-        <v>45915</v>
-      </c>
-      <c r="G4" s="12" cm="1">
-        <f t="array" ref="G4">G3+7</f>
-        <v>46290</v>
-      </c>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="18"/>
-    </row>
-    <row r="5" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B5" s="16" t="s">
+      <c r="C5" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="D5" s="65"/>
+      <c r="E5" s="9" cm="1">
+        <f t="array" ref="E5">E4+7</f>
+        <v>46297</v>
+      </c>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="15"/>
+    </row>
+    <row r="6" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="11" cm="1">
-        <f t="array" ref="F5">F4+7</f>
-        <v>45922</v>
-      </c>
-      <c r="G5" s="12" cm="1">
-        <f t="array" ref="G5">G4+7</f>
-        <v>46297</v>
-      </c>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="18"/>
-    </row>
-    <row r="6" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B6" s="16" t="s">
+      <c r="C6" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="D6" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="51" t="s">
+      <c r="E6" s="9" cm="1">
+        <f t="array" ref="E6">E5+7</f>
+        <v>46304</v>
+      </c>
+      <c r="F6" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="53"/>
-      <c r="F6" s="11" cm="1">
-        <f t="array" ref="F6">F5+7</f>
-        <v>45929</v>
-      </c>
-      <c r="G6" s="12" cm="1">
-        <f t="array" ref="G6">G5+7</f>
-        <v>46304</v>
-      </c>
-      <c r="H6" s="13" t="s">
+      <c r="G6" s="11"/>
+      <c r="H6" s="15"/>
+    </row>
+    <row r="7" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B7" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="14"/>
-      <c r="J6" s="18"/>
-    </row>
-    <row r="7" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B7" s="16" t="s">
+      <c r="C7" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="D7" s="65"/>
+      <c r="E7" s="9" cm="1">
+        <f t="array" ref="E7">E6+7</f>
+        <v>46311</v>
+      </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="15"/>
+    </row>
+    <row r="8" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B8" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52"/>
-      <c r="F7" s="11" cm="1">
-        <f t="array" ref="F7">F6+7</f>
-        <v>45936</v>
-      </c>
-      <c r="G7" s="12" cm="1">
-        <f t="array" ref="G7">G6+7</f>
-        <v>46311</v>
-      </c>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="18"/>
-    </row>
-    <row r="8" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B8" s="16" t="s">
+      <c r="C8" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="D8" s="65"/>
+      <c r="E8" s="9" cm="1">
+        <f t="array" ref="E8">E7+7</f>
+        <v>46318</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="15"/>
+    </row>
+    <row r="9" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B9" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="11" cm="1">
-        <f t="array" ref="F8">F7+7</f>
-        <v>45943</v>
-      </c>
-      <c r="G8" s="12" cm="1">
-        <f t="array" ref="G8">G7+7</f>
-        <v>46318</v>
-      </c>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="18"/>
-    </row>
-    <row r="9" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B9" s="16" t="s">
+      <c r="C9" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="D9" s="65"/>
+      <c r="E9" s="9" cm="1">
+        <f t="array" ref="E9">E8+7</f>
+        <v>46325</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="52"/>
-      <c r="E9" s="52"/>
-      <c r="F9" s="11" cm="1">
-        <f t="array" ref="F9">F8+7</f>
-        <v>45950</v>
-      </c>
-      <c r="G9" s="12" cm="1">
-        <f t="array" ref="G9">G8+7</f>
-        <v>46325</v>
-      </c>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="19" t="s">
+    </row>
+    <row r="10" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B10" s="13" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="10" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B10" s="16" t="s">
+      <c r="C10" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="D10" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="51" t="s">
+      <c r="E10" s="9" cm="1">
+        <f t="array" ref="E10">E9+7</f>
+        <v>46332</v>
+      </c>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" ht="44.7" customHeight="1">
+      <c r="B11" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="54"/>
-      <c r="F10" s="11" cm="1">
-        <f t="array" ref="F10">F9+7</f>
-        <v>45957</v>
-      </c>
-      <c r="G10" s="12" cm="1">
-        <f t="array" ref="G10">G9+7</f>
-        <v>46332</v>
-      </c>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="19" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" ht="44.7" customHeight="1">
-      <c r="B11" s="16" t="s">
+      <c r="C11" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="D11" s="65"/>
+      <c r="E11" s="9" cm="1">
+        <f t="array" ref="E11">E10+7</f>
+        <v>46339</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="52"/>
-      <c r="E11" s="55"/>
-      <c r="F11" s="11" cm="1">
-        <f t="array" ref="F11">F10+7</f>
-        <v>45964</v>
-      </c>
-      <c r="G11" s="12" cm="1">
-        <f t="array" ref="G11">G10+7</f>
-        <v>46339</v>
-      </c>
-      <c r="H11" s="13" t="s">
+      <c r="G11" s="11"/>
+      <c r="H11" s="15"/>
+    </row>
+    <row r="12" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B12" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="I11" s="14"/>
-      <c r="J11" s="18"/>
-    </row>
-    <row r="12" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B12" s="16" t="s">
+      <c r="C12" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="D12" s="65"/>
+      <c r="E12" s="9" cm="1">
+        <f t="array" ref="E12">E11+7</f>
+        <v>46346</v>
+      </c>
+      <c r="F12" s="15"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="15"/>
+    </row>
+    <row r="13" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B13" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="11" cm="1">
-        <f t="array" ref="F12">F11+7</f>
-        <v>45971</v>
-      </c>
-      <c r="G12" s="12" cm="1">
-        <f t="array" ref="G12">G11+7</f>
-        <v>46346</v>
-      </c>
-      <c r="H12" s="18"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="18"/>
-    </row>
-    <row r="13" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B13" s="16" t="s">
+      <c r="C13" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="D13" s="65"/>
+      <c r="E13" s="9" cm="1">
+        <f t="array" ref="E13">E12+7</f>
+        <v>46353</v>
+      </c>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="52"/>
-      <c r="E13" s="52"/>
-      <c r="F13" s="11" cm="1">
-        <f t="array" ref="F13">F12+7</f>
-        <v>45978</v>
-      </c>
-      <c r="G13" s="12" cm="1">
-        <f t="array" ref="G13">G12+7</f>
-        <v>46353</v>
-      </c>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="20" t="s">
+    </row>
+    <row r="14" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B14" s="13" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="14" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B14" s="16" t="s">
+      <c r="C14" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="D14" s="65"/>
+      <c r="E14" s="9" cm="1">
+        <f t="array" ref="E14">E13+7</f>
+        <v>46360</v>
+      </c>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="15"/>
+    </row>
+    <row r="15" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B15" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="52"/>
-      <c r="E14" s="52"/>
-      <c r="F14" s="11" cm="1">
-        <f t="array" ref="F14">F13+7</f>
-        <v>45985</v>
-      </c>
-      <c r="G14" s="12" cm="1">
-        <f t="array" ref="G14">G13+7</f>
-        <v>46360</v>
-      </c>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="18"/>
-    </row>
-    <row r="15" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B15" s="16" t="s">
+      <c r="C15" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="D15" s="64" t="s">
         <v>42</v>
       </c>
-      <c r="D15" s="51" t="s">
+      <c r="E15" s="9" cm="1">
+        <f t="array" ref="E15">E14+7</f>
+        <v>46367</v>
+      </c>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="53"/>
-      <c r="F15" s="11" cm="1">
-        <f t="array" ref="F15">F14+7</f>
-        <v>45992</v>
-      </c>
-      <c r="G15" s="12" cm="1">
-        <f t="array" ref="G15">G14+7</f>
-        <v>46367</v>
-      </c>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="19" t="s">
+    </row>
+    <row r="16" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B16" s="13" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="16" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B16" s="16" t="s">
+      <c r="C16" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="D16" s="65"/>
+      <c r="E16" s="9" cm="1">
+        <f t="array" ref="E16">E15+7</f>
+        <v>46374</v>
+      </c>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="52"/>
-      <c r="E16" s="52"/>
-      <c r="F16" s="11" cm="1">
-        <f t="array" ref="F16">F15+7</f>
-        <v>45999</v>
-      </c>
-      <c r="G16" s="12" cm="1">
-        <f t="array" ref="G16">G15+7</f>
-        <v>46374</v>
-      </c>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="21" t="s">
+    </row>
+    <row r="17" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B17" s="13" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="17" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B17" s="16" t="s">
+      <c r="C17" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="D17" s="65"/>
+      <c r="E17" s="9" cm="1">
+        <f t="array" ref="E17">E16+7</f>
+        <v>46381</v>
+      </c>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="52"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="11" cm="1">
-        <f t="array" ref="F17">F16+7</f>
-        <v>46006</v>
-      </c>
-      <c r="G17" s="12" cm="1">
-        <f t="array" ref="G17">G16+7</f>
-        <v>46381</v>
-      </c>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="19" t="s">
+    </row>
+    <row r="18" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B18" s="13" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="18" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B18" s="16" t="s">
+      <c r="C18" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="D18" s="65"/>
+      <c r="E18" s="9" cm="1">
+        <f t="array" ref="E18">E17+7</f>
+        <v>46388</v>
+      </c>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B19" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D18" s="52"/>
-      <c r="E18" s="52"/>
-      <c r="F18" s="11" cm="1">
-        <f t="array" ref="F18">F17+7</f>
-        <v>46013</v>
-      </c>
-      <c r="G18" s="12" cm="1">
-        <f t="array" ref="G18">G17+7</f>
-        <v>46388</v>
-      </c>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B19" s="16" t="s">
+      <c r="C19" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="D19" s="64" t="s">
         <v>54</v>
       </c>
-      <c r="D19" s="51" t="s">
+      <c r="E19" s="9" cm="1">
+        <f t="array" ref="E19">E18+7</f>
+        <v>46395</v>
+      </c>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B20" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="52"/>
-      <c r="F19" s="11" cm="1">
-        <f t="array" ref="F19">F18+7</f>
-        <v>46020</v>
-      </c>
-      <c r="G19" s="12" cm="1">
-        <f t="array" ref="G19">G18+7</f>
-        <v>46395</v>
-      </c>
-      <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B20" s="22" t="s">
+      <c r="C20" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="D20" s="65"/>
+      <c r="E20" s="9" cm="1">
+        <f t="array" ref="E20">E19+7</f>
+        <v>46402</v>
+      </c>
+      <c r="F20" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="52"/>
-      <c r="E20" s="53"/>
-      <c r="F20" s="11" cm="1">
-        <f t="array" ref="F20">F19+7</f>
-        <v>46027</v>
-      </c>
-      <c r="G20" s="12" cm="1">
-        <f t="array" ref="G20">G19+7</f>
-        <v>46402</v>
-      </c>
-      <c r="H20" s="13" t="s">
+      <c r="G20" s="11"/>
+      <c r="H20" s="15"/>
+    </row>
+    <row r="21" spans="2:8" ht="45.75" customHeight="1">
+      <c r="B21" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="I20" s="14"/>
-      <c r="J20" s="18"/>
-    </row>
-    <row r="21" spans="2:10" ht="45.75" customHeight="1">
-      <c r="B21" s="24" t="s">
+      <c r="C21" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C21" s="25" t="s">
+      <c r="D21" s="65"/>
+      <c r="E21" s="23" cm="1">
+        <f t="array" ref="E21">E20+7</f>
+        <v>46409</v>
+      </c>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="D21" s="52"/>
-      <c r="E21" s="52"/>
-      <c r="F21" s="11" cm="1">
-        <f t="array" ref="F21">F20+7</f>
-        <v>46034</v>
-      </c>
-      <c r="G21" s="26" cm="1">
-        <f t="array" ref="G21">G20+7</f>
-        <v>46409</v>
-      </c>
-      <c r="H21" s="27"/>
-      <c r="I21" s="27"/>
-      <c r="J21" s="28" t="s">
+    </row>
+    <row r="22" spans="2:8" ht="21.75" customHeight="1">
+      <c r="B22" s="13" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="22" spans="2:10" ht="21.75" customHeight="1">
-      <c r="B22" s="16" t="s">
+      <c r="C22" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="D22" s="65"/>
+      <c r="E22" s="26" cm="1">
+        <f t="array" ref="E22">E21+7</f>
+        <v>46416</v>
+      </c>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="11" cm="1">
-        <f t="array" ref="F22">F21+7</f>
-        <v>46041</v>
-      </c>
-      <c r="G22" s="29" cm="1">
-        <f t="array" ref="G22">G21+7</f>
-        <v>46416</v>
-      </c>
-      <c r="H22" s="30"/>
-      <c r="I22" s="30"/>
-      <c r="J22" s="31" t="s">
+    </row>
+    <row r="23" spans="2:8" ht="21.15" customHeight="1">
+      <c r="B23" s="29" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="23" spans="2:10" ht="21.15" customHeight="1">
-      <c r="B23" s="32" t="s">
+      <c r="C23" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="33" t="s">
+      <c r="D23" s="66" t="s">
         <v>66</v>
       </c>
-      <c r="D23" s="56" t="s">
+      <c r="E23" s="9" cm="1">
+        <f t="array" ref="E23">E22+7</f>
+        <v>46423</v>
+      </c>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="E23" s="52"/>
-      <c r="F23" s="11" cm="1">
-        <f t="array" ref="F23">F22+7</f>
-        <v>46048</v>
-      </c>
-      <c r="G23" s="12" cm="1">
-        <f t="array" ref="G23">G22+7</f>
-        <v>46423</v>
-      </c>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="19" t="s">
+    </row>
+    <row r="24" spans="2:8" ht="33.15" customHeight="1">
+      <c r="B24" s="31" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="24" spans="2:10" ht="33.15" customHeight="1">
-      <c r="B24" s="34" t="s">
+      <c r="C24" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="C24" s="35" t="s">
+      <c r="D24" s="65"/>
+      <c r="E24" s="9" cm="1">
+        <f t="array" ref="E24">E23+7</f>
+        <v>46430</v>
+      </c>
+      <c r="F24" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="D24" s="52"/>
-      <c r="E24" s="53"/>
-      <c r="F24" s="11" cm="1">
-        <f t="array" ref="F24">F23+7</f>
-        <v>46055</v>
-      </c>
-      <c r="G24" s="12" cm="1">
-        <f t="array" ref="G24">G23+7</f>
-        <v>46430</v>
-      </c>
-      <c r="H24" s="36" t="s">
+      <c r="G24" s="11"/>
+      <c r="H24" s="15"/>
+    </row>
+    <row r="25" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B25" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="I24" s="14"/>
-      <c r="J24" s="18"/>
-    </row>
-    <row r="25" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B25" s="16" t="s">
+      <c r="C25" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="D25" s="65"/>
+      <c r="E25" s="9" cm="1">
+        <f t="array" ref="E25">E24+7</f>
+        <v>46437</v>
+      </c>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="15"/>
+    </row>
+    <row r="26" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B26" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D25" s="52"/>
-      <c r="E25" s="52"/>
-      <c r="F25" s="37" cm="1">
-        <f t="array" ref="F25">F24+7</f>
-        <v>46062</v>
-      </c>
-      <c r="G25" s="12" cm="1">
-        <f t="array" ref="G25">G24+7</f>
-        <v>46437</v>
-      </c>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="18"/>
-    </row>
-    <row r="26" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B26" s="16" t="s">
+      <c r="C26" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="D26" s="65"/>
+      <c r="E26" s="9" cm="1">
+        <f t="array" ref="E26">E25+7</f>
+        <v>46444</v>
+      </c>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="15"/>
+    </row>
+    <row r="27" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B27" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="D26" s="52"/>
-      <c r="E26" s="52"/>
-      <c r="F26" s="38" cm="1">
-        <f t="array" ref="F26">F25+7</f>
-        <v>46069</v>
-      </c>
-      <c r="G26" s="12" cm="1">
-        <f t="array" ref="G26">G25+7</f>
-        <v>46444</v>
-      </c>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="18"/>
-    </row>
-    <row r="27" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B27" s="16" t="s">
+      <c r="C27" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="D27" s="64" t="s">
         <v>77</v>
       </c>
-      <c r="D27" s="51" t="s">
+      <c r="E27" s="9" cm="1">
+        <f t="array" ref="E27">E26+7</f>
+        <v>46451</v>
+      </c>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="15"/>
+    </row>
+    <row r="28" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B28" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="E27" s="52"/>
-      <c r="F27" s="11" cm="1">
-        <f t="array" ref="F27">F26+7</f>
-        <v>46076</v>
-      </c>
-      <c r="G27" s="12" cm="1">
-        <f t="array" ref="G27">G26+7</f>
-        <v>46451</v>
-      </c>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="18"/>
-    </row>
-    <row r="28" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B28" s="16" t="s">
+      <c r="C28" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="D28" s="65"/>
+      <c r="E28" s="9" cm="1">
+        <f t="array" ref="E28">E27+7</f>
+        <v>46458</v>
+      </c>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="15"/>
+    </row>
+    <row r="29" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B29" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="D28" s="52"/>
-      <c r="E28" s="53"/>
-      <c r="F28" s="11" cm="1">
-        <f t="array" ref="F28">F27+7</f>
-        <v>46083</v>
-      </c>
-      <c r="G28" s="12" cm="1">
-        <f t="array" ref="G28">G27+7</f>
-        <v>46458</v>
-      </c>
-      <c r="H28" s="14"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="18"/>
-    </row>
-    <row r="29" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B29" s="16" t="s">
+      <c r="C29" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="D29" s="65"/>
+      <c r="E29" s="9" cm="1">
+        <f t="array" ref="E29">E28+7</f>
+        <v>46465</v>
+      </c>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="15"/>
+    </row>
+    <row r="30" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B30" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="D29" s="52"/>
-      <c r="E29" s="52"/>
-      <c r="F29" s="11" cm="1">
-        <f t="array" ref="F29">F28+7</f>
-        <v>46090</v>
-      </c>
-      <c r="G29" s="12" cm="1">
-        <f t="array" ref="G29">G28+7</f>
-        <v>46465</v>
-      </c>
-      <c r="H29" s="14"/>
-      <c r="I29" s="14"/>
-      <c r="J29" s="18"/>
-    </row>
-    <row r="30" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B30" s="16" t="s">
+      <c r="C30" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="D30" s="65"/>
+      <c r="E30" s="9" cm="1">
+        <f t="array" ref="E30">E29+7</f>
+        <v>46472</v>
+      </c>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="D30" s="52"/>
-      <c r="E30" s="52"/>
-      <c r="F30" s="11" cm="1">
-        <f t="array" ref="F30">F29+7</f>
-        <v>46097</v>
-      </c>
-      <c r="G30" s="12" cm="1">
-        <f t="array" ref="G30">G29+7</f>
-        <v>46472</v>
-      </c>
-      <c r="H30" s="14"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="19" t="s">
+    </row>
+    <row r="31" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B31" s="13" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="31" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B31" s="16" t="s">
+      <c r="C31" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="D31" s="65"/>
+      <c r="E31" s="9" cm="1">
+        <f t="array" ref="E31">E30+7</f>
+        <v>46479</v>
+      </c>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B32" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="D31" s="52"/>
-      <c r="E31" s="52"/>
-      <c r="F31" s="11" cm="1">
-        <f t="array" ref="F31">F30+7</f>
-        <v>46104</v>
-      </c>
-      <c r="G31" s="12" cm="1">
-        <f t="array" ref="G31">G30+7</f>
-        <v>46479</v>
-      </c>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="19" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="32" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B32" s="16" t="s">
+      <c r="C32" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="C32" s="17" t="s">
+      <c r="D32" s="64" t="s">
         <v>89</v>
       </c>
-      <c r="D32" s="51" t="s">
+      <c r="E32" s="9" cm="1">
+        <f t="array" ref="E32">E31+7</f>
+        <v>46486</v>
+      </c>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="15"/>
+    </row>
+    <row r="33" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B33" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="E32" s="53"/>
-      <c r="F32" s="11" cm="1">
-        <f t="array" ref="F32">F31+7</f>
-        <v>46111</v>
-      </c>
-      <c r="G32" s="12" cm="1">
-        <f t="array" ref="G32">G31+7</f>
-        <v>46486</v>
-      </c>
-      <c r="H32" s="14"/>
-      <c r="I32" s="14"/>
-      <c r="J32" s="18"/>
-    </row>
-    <row r="33" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B33" s="16" t="s">
+      <c r="C33" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="D33" s="65"/>
+      <c r="E33" s="9" cm="1">
+        <f t="array" ref="E33">E32+7</f>
+        <v>46493</v>
+      </c>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="D33" s="52"/>
-      <c r="E33" s="52"/>
-      <c r="F33" s="11" cm="1">
-        <f t="array" ref="F33">F32+7</f>
-        <v>46118</v>
-      </c>
-      <c r="G33" s="12" cm="1">
-        <f t="array" ref="G33">G32+7</f>
-        <v>46493</v>
-      </c>
-      <c r="H33" s="14"/>
-      <c r="I33" s="14"/>
-      <c r="J33" s="19" t="s">
+    </row>
+    <row r="34" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B34" s="13" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="34" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B34" s="16" t="s">
+      <c r="C34" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="D34" s="65"/>
+      <c r="E34" s="9" cm="1">
+        <f t="array" ref="E34">E33+7</f>
+        <v>46500</v>
+      </c>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="15"/>
+    </row>
+    <row r="35" spans="2:8" ht="44.7" customHeight="1">
+      <c r="B35" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="D34" s="52"/>
-      <c r="E34" s="52"/>
-      <c r="F34" s="11" cm="1">
-        <f t="array" ref="F34">F33+7</f>
-        <v>46125</v>
-      </c>
-      <c r="G34" s="12" cm="1">
-        <f t="array" ref="G34">G33+7</f>
-        <v>46500</v>
-      </c>
-      <c r="H34" s="14"/>
-      <c r="I34" s="14"/>
-      <c r="J34" s="18"/>
-    </row>
-    <row r="35" spans="2:10" ht="44.7" customHeight="1">
-      <c r="B35" s="16" t="s">
+      <c r="C35" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="C35" s="17" t="s">
+      <c r="D35" s="65"/>
+      <c r="E35" s="9" cm="1">
+        <f t="array" ref="E35">E34+7</f>
+        <v>46507</v>
+      </c>
+      <c r="F35" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="D35" s="52"/>
-      <c r="E35" s="52"/>
-      <c r="F35" s="11" cm="1">
-        <f t="array" ref="F35">F34+7</f>
-        <v>46132</v>
-      </c>
-      <c r="G35" s="12" cm="1">
-        <f t="array" ref="G35">G34+7</f>
-        <v>46507</v>
-      </c>
-      <c r="H35" s="13" t="s">
+      <c r="G35" s="11"/>
+      <c r="H35" s="15"/>
+    </row>
+    <row r="36" spans="2:8" ht="44.7" customHeight="1">
+      <c r="B36" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="I35" s="14"/>
-      <c r="J35" s="18"/>
-    </row>
-    <row r="36" spans="2:10" ht="44.7" customHeight="1">
-      <c r="B36" s="16" t="s">
+      <c r="C36" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="C36" s="17" t="s">
+      <c r="D36" s="64" t="s">
         <v>100</v>
       </c>
-      <c r="D36" s="51" t="s">
+      <c r="E36" s="9" cm="1">
+        <f t="array" ref="E36">E35+7</f>
+        <v>46514</v>
+      </c>
+      <c r="F36" s="11"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="E36" s="52"/>
-      <c r="F36" s="11" cm="1">
-        <f t="array" ref="F36">F35+7</f>
-        <v>46139</v>
-      </c>
-      <c r="G36" s="12" cm="1">
-        <f t="array" ref="G36">G35+7</f>
-        <v>46514</v>
-      </c>
-      <c r="H36" s="14"/>
-      <c r="I36" s="14"/>
-      <c r="J36" s="21" t="s">
+    </row>
+    <row r="37" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B37" s="13" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="37" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B37" s="16" t="s">
+      <c r="C37" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="C37" s="17" t="s">
+      <c r="D37" s="65"/>
+      <c r="E37" s="9" cm="1">
+        <f t="array" ref="E37">E36+7</f>
+        <v>46521</v>
+      </c>
+      <c r="F37" s="11"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="15"/>
+    </row>
+    <row r="38" spans="2:8" ht="21.75" customHeight="1">
+      <c r="B38" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="D37" s="52"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="11" cm="1">
-        <f t="array" ref="F37">F36+7</f>
-        <v>46146</v>
-      </c>
-      <c r="G37" s="12" cm="1">
-        <f t="array" ref="G37">G36+7</f>
-        <v>46521</v>
-      </c>
-      <c r="H37" s="14"/>
-      <c r="I37" s="14"/>
-      <c r="J37" s="18"/>
-    </row>
-    <row r="38" spans="2:10" ht="21.75" customHeight="1">
-      <c r="B38" s="16" t="s">
+      <c r="C38" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="C38" s="17" t="s">
+      <c r="D38" s="65"/>
+      <c r="E38" s="34" cm="1">
+        <f t="array" ref="E38">E37+7</f>
+        <v>46528</v>
+      </c>
+      <c r="F38" s="35"/>
+      <c r="G38" s="35"/>
+      <c r="H38" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="D38" s="52"/>
-      <c r="E38" s="52"/>
-      <c r="F38" s="11" cm="1">
-        <f t="array" ref="F38">F37+7</f>
-        <v>46153</v>
-      </c>
-      <c r="G38" s="39" cm="1">
-        <f t="array" ref="G38">G37+7</f>
-        <v>46528</v>
-      </c>
-      <c r="H38" s="40"/>
-      <c r="I38" s="40"/>
-      <c r="J38" s="41" t="s">
+    </row>
+    <row r="39" spans="2:8" ht="67.95" customHeight="1">
+      <c r="B39" s="13" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="39" spans="2:10" ht="67.95" customHeight="1">
-      <c r="B39" s="16" t="s">
+      <c r="C39" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="C39" s="17" t="s">
+      <c r="D39" s="65"/>
+      <c r="E39" s="37" cm="1">
+        <f t="array" ref="E39">E38+7</f>
+        <v>46535</v>
+      </c>
+      <c r="F39" s="38"/>
+      <c r="G39" s="39"/>
+      <c r="H39" s="40" t="s">
         <v>109</v>
       </c>
-      <c r="D39" s="52"/>
-      <c r="E39" s="52"/>
-      <c r="F39" s="11" cm="1">
-        <f t="array" ref="F39">F38+7</f>
-        <v>46160</v>
-      </c>
-      <c r="G39" s="42" cm="1">
-        <f t="array" ref="G39">G38+7</f>
-        <v>46535</v>
-      </c>
-      <c r="H39" s="43"/>
-      <c r="I39" s="44"/>
-      <c r="J39" s="45" t="s">
+    </row>
+    <row r="40" spans="2:8" ht="32.700000000000003" customHeight="1">
+      <c r="B40" s="13" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="40" spans="2:10" ht="32.700000000000003" customHeight="1">
-      <c r="B40" s="16" t="s">
+      <c r="C40" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="C40" s="17" t="s">
+      <c r="D40" s="65"/>
+      <c r="E40" s="9" cm="1">
+        <f t="array" ref="E40">E39+7</f>
+        <v>46542</v>
+      </c>
+      <c r="F40" s="33" t="s">
         <v>112</v>
       </c>
-      <c r="D40" s="52"/>
-      <c r="E40" s="52"/>
-      <c r="F40" s="11" cm="1">
-        <f t="array" ref="F40">F39+7</f>
-        <v>46167</v>
-      </c>
-      <c r="G40" s="12" cm="1">
-        <f t="array" ref="G40">G39+7</f>
-        <v>46542</v>
-      </c>
-      <c r="H40" s="36" t="s">
+      <c r="G40" s="11"/>
+      <c r="H40" s="15"/>
+    </row>
+    <row r="41" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B41" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="I40" s="14"/>
-      <c r="J40" s="18"/>
-    </row>
-    <row r="41" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B41" s="16" t="s">
+      <c r="C41" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="D41" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="D41" s="51" t="s">
+      <c r="E41" s="9" cm="1">
+        <f t="array" ref="E41">E40+7</f>
+        <v>46549</v>
+      </c>
+      <c r="F41" s="11"/>
+      <c r="G41" s="11"/>
+      <c r="H41" s="15"/>
+    </row>
+    <row r="42" spans="2:8" ht="45.75" customHeight="1">
+      <c r="B42" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="E41" s="55"/>
-      <c r="F41" s="11" cm="1">
-        <f t="array" ref="F41">F40+7</f>
-        <v>46174</v>
-      </c>
-      <c r="G41" s="12" cm="1">
-        <f t="array" ref="G41">G40+7</f>
-        <v>46549</v>
-      </c>
-      <c r="H41" s="14"/>
-      <c r="I41" s="14"/>
-      <c r="J41" s="18"/>
-    </row>
-    <row r="42" spans="2:10" ht="45.75" customHeight="1">
-      <c r="B42" s="16" t="s">
+      <c r="C42" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="C42" s="17" t="s">
+      <c r="D42" s="65"/>
+      <c r="E42" s="23" cm="1">
+        <f t="array" ref="E42">E41+7</f>
+        <v>46556</v>
+      </c>
+      <c r="F42" s="24"/>
+      <c r="G42" s="24"/>
+      <c r="H42" s="41" t="s">
         <v>118</v>
       </c>
-      <c r="D42" s="52"/>
-      <c r="E42" s="52"/>
-      <c r="F42" s="11" cm="1">
-        <f t="array" ref="F42">F41+7</f>
-        <v>46181</v>
-      </c>
-      <c r="G42" s="26" cm="1">
-        <f t="array" ref="G42">G41+7</f>
-        <v>46556</v>
-      </c>
-      <c r="H42" s="27"/>
-      <c r="I42" s="27"/>
-      <c r="J42" s="46" t="s">
+    </row>
+    <row r="43" spans="2:8" ht="21.75" customHeight="1">
+      <c r="B43" s="13" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="43" spans="2:10" ht="21.75" customHeight="1">
-      <c r="B43" s="16" t="s">
+      <c r="C43" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="C43" s="17" t="s">
+      <c r="D43" s="65"/>
+      <c r="E43" s="26" cm="1">
+        <f t="array" ref="E43">E42+7</f>
+        <v>46563</v>
+      </c>
+      <c r="F43" s="42"/>
+      <c r="G43" s="42"/>
+      <c r="H43" s="43" t="s">
         <v>121</v>
       </c>
-      <c r="D43" s="52"/>
-      <c r="E43" s="52"/>
-      <c r="F43" s="11" cm="1">
-        <f t="array" ref="F43">F42+7</f>
-        <v>46188</v>
-      </c>
-      <c r="G43" s="29" cm="1">
-        <f t="array" ref="G43">G42+7</f>
-        <v>46563</v>
-      </c>
-      <c r="H43" s="47"/>
-      <c r="I43" s="47"/>
-      <c r="J43" s="48" t="s">
+    </row>
+    <row r="44" spans="2:8" ht="68.7" customHeight="1">
+      <c r="B44" s="13" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="44" spans="2:10" ht="68.7" customHeight="1">
-      <c r="B44" s="16" t="s">
+      <c r="C44" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="C44" s="17" t="s">
+      <c r="D44" s="65"/>
+      <c r="E44" s="9" cm="1">
+        <f t="array" ref="E44">E43+7</f>
+        <v>46570</v>
+      </c>
+      <c r="F44" s="11"/>
+      <c r="G44" s="11"/>
+      <c r="H44" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="D44" s="52"/>
-      <c r="E44" s="52"/>
-      <c r="F44" s="11" cm="1">
-        <f t="array" ref="F44">F43+7</f>
-        <v>46195</v>
-      </c>
-      <c r="G44" s="12" cm="1">
-        <f t="array" ref="G44">G43+7</f>
-        <v>46570</v>
-      </c>
-      <c r="H44" s="14"/>
-      <c r="I44" s="14"/>
-      <c r="J44" s="49" t="s">
+    </row>
+    <row r="45" spans="2:8" ht="20.7" customHeight="1">
+      <c r="B45" s="13" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="45" spans="2:10" ht="20.7" customHeight="1">
-      <c r="B45" s="16" t="s">
+      <c r="C45" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="C45" s="17" t="s">
-        <v>127</v>
-      </c>
-      <c r="D45" s="50">
+      <c r="D45" s="45">
         <v>46204</v>
       </c>
-      <c r="E45" s="52"/>
-      <c r="F45" s="11" cm="1">
-        <f t="array" ref="F45">F44+7</f>
-        <v>46202</v>
-      </c>
-      <c r="G45" s="12" cm="1">
-        <f t="array" ref="G45">G44+7</f>
+      <c r="E45" s="9" cm="1">
+        <f t="array" ref="E45">E44+7</f>
         <v>46577</v>
       </c>
-      <c r="H45" s="14"/>
-      <c r="I45" s="14"/>
-      <c r="J45" s="18"/>
+      <c r="F45" s="11"/>
+      <c r="G45" s="11"/>
+      <c r="H45" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="E41:E45"/>
-    <mergeCell ref="D6:D9"/>
-    <mergeCell ref="D10:D14"/>
-    <mergeCell ref="D15:D18"/>
-    <mergeCell ref="D19:D22"/>
+  <mergeCells count="10">
     <mergeCell ref="D23:D26"/>
     <mergeCell ref="D27:D31"/>
     <mergeCell ref="D32:D35"/>
     <mergeCell ref="D36:D40"/>
     <mergeCell ref="D41:D44"/>
-    <mergeCell ref="E20:E23"/>
-    <mergeCell ref="E24:E27"/>
-    <mergeCell ref="E28:E31"/>
-    <mergeCell ref="E32:E36"/>
-    <mergeCell ref="E37:E40"/>
     <mergeCell ref="D2:D5"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="E6:E10"/>
-    <mergeCell ref="E11:E14"/>
-    <mergeCell ref="E15:E19"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="D10:D14"/>
+    <mergeCell ref="D15:D18"/>
+    <mergeCell ref="D19:D22"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="I2" r:id="rId1" xr:uid="{05B5B872-5477-4A6E-8248-74AD138D28B6}"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{05B5B872-5477-4A6E-8248-74AD138D28B6}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{20589D99-E2C2-493B-BCF0-A1BAD54E5F0E}"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup scale="55" orientation="portrait"/>

</xml_diff>